<commit_message>
docs: add SyslogNG bid workbook and risk scoring guide
</commit_message>
<xml_diff>
--- a/projects/syslog-ng-centralized-logging/bid-estimate/SyslogNG-Upwork-Bid-Feasibility-and-Cost-Estimate.xlsx
+++ b/projects/syslog-ng-centralized-logging/bid-estimate/SyslogNG-Upwork-Bid-Feasibility-and-Cost-Estimate.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bid Summary" sheetId="1" r:id="R06f81d3e35a94816"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Work Breakdown" sheetId="2" r:id="R63b1491dd6c04c03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing Calculator" sheetId="3" r:id="R6c80181b8c5b4881"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="4" r:id="Rf8beb40edcda4cfb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions &amp; Questions" sheetId="5" r:id="R9ebb81952fd24178"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="6" r:id="R683ee69db2b24246"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Criteria" sheetId="7" r:id="R0989e036bdf54de4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bid Summary" sheetId="1" r:id="R79fd70d6001f40cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Work Breakdown" sheetId="2" r:id="R0e4ee70f23b2457f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing Calculator" sheetId="3" r:id="Rd140025f615e49db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="4" r:id="Rf414e3df059b4e69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions &amp; Questions" sheetId="5" r:id="R97ad3957c3e94e61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="6" r:id="Rf595b25ae1654801"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Criteria" sheetId="7" r:id="R9604d1823d884b08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Scoring Guide" sheetId="8" r:id="Rbdb4df7fb79b4523"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -33,6 +34,70 @@
 </x:comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:authors>
+    <x:author>tc={236E16AE-CE35-66D5-C8B8-23FB2523AE8B}</x:author>
+    <x:author>tc={71340E2D-985B-C86F-A7DE-A0CC60BF581B}</x:author>
+    <x:author>tc={ECBDA878-B225-1BAC-83D0-062B923933B4}</x:author>
+    <x:author>tc={0C3B199A-314C-C12C-D924-4FE7EB03CFFD}</x:author>
+    <x:author>tc={F24977D6-6CBB-E302-8C35-2821A8CC92FD}</x:author>
+  </x:authors>
+  <x:commentList>
+    <x:comment ref="C4" authorId="0">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Probability: the likelihood that the risk will occur. Rate from 1 (Rare) to 5 (Almost certain).</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="D4" authorId="1">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Impact: the severity of the effect if the risk occurs. Rate from 1 (Insignificant) to 5 (Critical).</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="E4" authorId="2">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Score: Probability multiplied by Impact. The result ranges from 1 to 25.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="F4" authorId="3">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Mitigation: the action planned to reduce the probability, impact, or both.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="G4" authorId="4">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Owner: the person or party responsible for monitoring and managing the risk.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+  </x:commentList>
+</x:comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
@@ -45,7 +110,7 @@
     <x:numFmt numFmtId="202" formatCode="0%"/>
     <x:numFmt numFmtId="203" formatCode="&quot;$&quot;#,##0.00"/>
   </x:numFmts>
-  <x:fonts count="22">
+  <x:fonts count="44">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -170,8 +235,135 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F1F1F"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF404040"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF404040"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF375623"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="18"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF404040"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF404040"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF375623"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF404040"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF375623"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="19">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -218,8 +410,53 @@
         <x:fgColor rgb="FF70AD47"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F75B5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4CCCC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="23">
+  <x:borders count="32">
     <x:border/>
     <x:border>
       <x:left style="medium">
@@ -397,11 +634,77 @@
         <x:color rgb="FF70AD47"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF9EADBA"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FF9EADBA"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FF9EADBA"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FF9EADBA"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF9EADBA"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF9EADBA"/>
+      </x:left>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FF9EADBA"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF9EADBA"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FF9EADBA"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FF9EADBA"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FF9EADBA"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FF9EADBA"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="220">
+  <x:cellXfs count="332">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -922,6 +1225,284 @@
     <x:xf numFmtId="0" fontId="19" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="11" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="11" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="24" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="25" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="11" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="11" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="15" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="15" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="29" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="30" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="33" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="34" fillId="11" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="14" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="14" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="35" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="34" fillId="11" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="16" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="16" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="37" fillId="15" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="15" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="15" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="17" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="17" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="18" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="18" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="14" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="14" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="40" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="11" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="41" fillId="11" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="16" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="16" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="42" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="40" fillId="15" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="15" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="15" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="17" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="17" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="18" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="18" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="43" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -933,7 +1514,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -944,7 +1525,7 @@
         <x:color rgb="FFC00000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -955,7 +1536,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -966,7 +1547,7 @@
         <x:color rgb="FFC00000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -977,7 +1558,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -988,7 +1569,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -999,7 +1580,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1010,7 +1591,7 @@
         <x:color rgb="FFC00000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -1022,6 +1603,7 @@
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
   <xltc:person displayName="Muhammad Khalid Khan" id="{8A082B11-3B6F-4306-87D9-09463CBE6C56}"/>
+  <xltc:person displayName="Muhammad Khalid Khan" id="{2DFB9B77-C8CF-46CB-88AB-1C16C7A2222E}"/>
 </xltc:personList>
 </file>
 
@@ -1224,6 +1806,26 @@
 </xltc:ThreadedComments>
 </file>
 
+<file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
+<xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <xltc:threadedComment ref="C4" dT="2026-07-16T16:55:32.831" personId="{2DFB9B77-C8CF-46CB-88AB-1C16C7A2222E}" id="{236E16AE-CE35-66D5-C8B8-23FB2523AE8B}">
+    <xltc:text>Probability: the likelihood that the risk will occur. Rate from 1 (Rare) to 5 (Almost certain).</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="D4" dT="2026-07-16T16:55:32.831" personId="{2DFB9B77-C8CF-46CB-88AB-1C16C7A2222E}" id="{71340E2D-985B-C86F-A7DE-A0CC60BF581B}">
+    <xltc:text>Impact: the severity of the effect if the risk occurs. Rate from 1 (Insignificant) to 5 (Critical).</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="E4" dT="2026-07-16T16:55:32.831" personId="{2DFB9B77-C8CF-46CB-88AB-1C16C7A2222E}" id="{ECBDA878-B225-1BAC-83D0-062B923933B4}">
+    <xltc:text>Score: Probability multiplied by Impact. The result ranges from 1 to 25.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="F4" dT="2026-07-16T16:55:32.831" personId="{2DFB9B77-C8CF-46CB-88AB-1C16C7A2222E}" id="{0C3B199A-314C-C12C-D924-4FE7EB03CFFD}">
+    <xltc:text>Mitigation: the action planned to reduce the probability, impact, or both.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="G4" dT="2026-07-16T16:55:32.831" personId="{2DFB9B77-C8CF-46CB-88AB-1C16C7A2222E}" id="{F24977D6-6CBB-E302-8C35-2821A8CC92FD}">
+    <xltc:text>Owner: the person or party responsible for monitoring and managing the risk.</xltc:text>
+  </xltc:threadedComment>
+</xltc:ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -2440,7 +3042,7 @@
     <x:mergeCell ref="D4:F4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12ad04f2c5f74a7e"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc814d5ffdc240e2"/>
 </x:worksheet>
 </file>
 
@@ -3466,9 +4068,45 @@
         <x:v>Client</x:v>
       </x:c>
     </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="231" t="str">
+        <x:v>HOW TO READ THE RISK SCORE</x:v>
+      </x:c>
+      <x:c r="B14" s="232"/>
+      <x:c r="C14" s="232"/>
+      <x:c r="D14" s="232"/>
+      <x:c r="E14" s="232"/>
+      <x:c r="F14" s="232"/>
+      <x:c r="G14" s="233"/>
+    </x:row>
+    <x:row r="15" ht="34" customHeight="1">
+      <x:c r="A15" s="234" t="str">
+        <x:v>Probability and Impact are rated from 1 to 5. Risk Score = Probability × Impact. A higher score requires stronger and faster mitigation.</x:v>
+      </x:c>
+      <x:c r="B15" s="235"/>
+      <x:c r="C15" s="235"/>
+      <x:c r="D15" s="235"/>
+      <x:c r="E15" s="235"/>
+      <x:c r="F15" s="235"/>
+      <x:c r="G15" s="236"/>
+    </x:row>
+    <x:row r="16" ht="32" customHeight="1">
+      <x:c r="A16" s="237" t="str">
+        <x:v>Score levels: 1–4 Low | 5–9 Medium | 10–14 High | 15–25 Critical. See the ‘Risk Scoring Guide’ worksheet for definitions and an example.</x:v>
+      </x:c>
+      <x:c r="B16" s="238"/>
+      <x:c r="C16" s="238"/>
+      <x:c r="D16" s="238"/>
+      <x:c r="E16" s="238"/>
+      <x:c r="F16" s="238"/>
+      <x:c r="G16" s="239"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G2"/>
+    <x:mergeCell ref="A14:G14"/>
+    <x:mergeCell ref="A15:G15"/>
+    <x:mergeCell ref="A16:G16"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="E5:E12">
     <x:cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThanOrEqual">
@@ -3489,6 +4127,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71c4bc475b9e494a"/>
 </x:worksheet>
 </file>
 
@@ -3770,4 +4409,441 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="31" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="25" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="291" t="str">
+        <x:v>RISK SCORING GUIDE</x:v>
+      </x:c>
+      <x:c r="B1" s="291"/>
+      <x:c r="C1" s="291"/>
+      <x:c r="D1" s="291"/>
+      <x:c r="E1" s="291"/>
+      <x:c r="F1" s="291"/>
+      <x:c r="G1" s="291"/>
+      <x:c r="H1" s="291"/>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="291"/>
+      <x:c r="B2" s="291"/>
+      <x:c r="C2" s="291"/>
+      <x:c r="D2" s="291"/>
+      <x:c r="E2" s="291"/>
+      <x:c r="F2" s="291"/>
+      <x:c r="G2" s="291"/>
+      <x:c r="H2" s="291"/>
+    </x:row>
+    <x:row r="3" ht="24" customHeight="1">
+      <x:c r="A3" s="292" t="str">
+        <x:v>Use this guide to assess, prioritize and explain the risks recorded in the Risks worksheet.</x:v>
+      </x:c>
+      <x:c r="B3" s="292"/>
+      <x:c r="C3" s="292"/>
+      <x:c r="D3" s="292"/>
+      <x:c r="E3" s="292"/>
+      <x:c r="F3" s="292"/>
+      <x:c r="G3" s="292"/>
+      <x:c r="H3" s="292"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="293"/>
+      <x:c r="B4" s="293"/>
+      <x:c r="C4" s="293"/>
+      <x:c r="D4" s="293"/>
+      <x:c r="E4" s="293"/>
+      <x:c r="F4" s="293"/>
+      <x:c r="G4" s="293"/>
+      <x:c r="H4" s="293"/>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="294" t="str">
+        <x:v>PROBABILITY — LIKELIHOOD OF OCCURRENCE</x:v>
+      </x:c>
+      <x:c r="B5" s="294"/>
+      <x:c r="C5" s="294"/>
+      <x:c r="D5" s="294" t="str">
+        <x:v>IMPACT — SEVERITY IF IT OCCURS</x:v>
+      </x:c>
+      <x:c r="E5" s="294"/>
+      <x:c r="F5" s="294"/>
+      <x:c r="G5" s="293"/>
+      <x:c r="H5" s="293"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="295" t="str">
+        <x:v>Rating</x:v>
+      </x:c>
+      <x:c r="B6" s="295" t="str">
+        <x:v>Level</x:v>
+      </x:c>
+      <x:c r="C6" s="295" t="str">
+        <x:v>Meaning</x:v>
+      </x:c>
+      <x:c r="D6" s="295" t="str">
+        <x:v>Rating</x:v>
+      </x:c>
+      <x:c r="E6" s="295" t="str">
+        <x:v>Level</x:v>
+      </x:c>
+      <x:c r="F6" s="295" t="str">
+        <x:v>Meaning</x:v>
+      </x:c>
+      <x:c r="G6" s="293"/>
+      <x:c r="H6" s="293"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="313" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B7" s="314" t="str">
+        <x:v>Rare</x:v>
+      </x:c>
+      <x:c r="C7" s="314" t="str">
+        <x:v>Very unlikely to occur</x:v>
+      </x:c>
+      <x:c r="D7" s="313" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E7" s="314" t="str">
+        <x:v>Insignificant</x:v>
+      </x:c>
+      <x:c r="F7" s="314" t="str">
+        <x:v>Little or no disruption</x:v>
+      </x:c>
+      <x:c r="G7" s="315"/>
+      <x:c r="H7" s="315"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="313" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B8" s="314" t="str">
+        <x:v>Unlikely</x:v>
+      </x:c>
+      <x:c r="C8" s="314" t="str">
+        <x:v>Could occur, but not expected</x:v>
+      </x:c>
+      <x:c r="D8" s="313" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E8" s="314" t="str">
+        <x:v>Minor</x:v>
+      </x:c>
+      <x:c r="F8" s="314" t="str">
+        <x:v>Small delay or limited rework</x:v>
+      </x:c>
+      <x:c r="G8" s="315"/>
+      <x:c r="H8" s="315"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="313" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B9" s="314" t="str">
+        <x:v>Possible</x:v>
+      </x:c>
+      <x:c r="C9" s="314" t="str">
+        <x:v>May occur during the project</x:v>
+      </x:c>
+      <x:c r="D9" s="313" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E9" s="314" t="str">
+        <x:v>Moderate</x:v>
+      </x:c>
+      <x:c r="F9" s="314" t="str">
+        <x:v>Noticeable cost, delay or service effect</x:v>
+      </x:c>
+      <x:c r="G9" s="315"/>
+      <x:c r="H9" s="315"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="313" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B10" s="314" t="str">
+        <x:v>Likely</x:v>
+      </x:c>
+      <x:c r="C10" s="314" t="str">
+        <x:v>Expected to occur in many cases</x:v>
+      </x:c>
+      <x:c r="D10" s="313" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E10" s="314" t="str">
+        <x:v>Major</x:v>
+      </x:c>
+      <x:c r="F10" s="314" t="str">
+        <x:v>Serious schedule, cost or service effect</x:v>
+      </x:c>
+      <x:c r="G10" s="315"/>
+      <x:c r="H10" s="315"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="313" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B11" s="314" t="str">
+        <x:v>Almost certain</x:v>
+      </x:c>
+      <x:c r="C11" s="314" t="str">
+        <x:v>Expected to occur or recur</x:v>
+      </x:c>
+      <x:c r="D11" s="313" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E11" s="314" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="F11" s="314" t="str">
+        <x:v>Severe outage, loss, compliance or evidence effect</x:v>
+      </x:c>
+      <x:c r="G11" s="315"/>
+      <x:c r="H11" s="315"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="315"/>
+      <x:c r="B12" s="315"/>
+      <x:c r="C12" s="315"/>
+      <x:c r="D12" s="315"/>
+      <x:c r="E12" s="315"/>
+      <x:c r="F12" s="315"/>
+      <x:c r="G12" s="315"/>
+      <x:c r="H12" s="315"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="294" t="str">
+        <x:v>CALCULATION METHOD</x:v>
+      </x:c>
+      <x:c r="B13" s="294"/>
+      <x:c r="C13" s="294"/>
+      <x:c r="D13" s="294"/>
+      <x:c r="E13" s="294"/>
+      <x:c r="F13" s="294"/>
+      <x:c r="G13" s="294"/>
+      <x:c r="H13" s="294"/>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="316" t="str">
+        <x:v>Risk Score = Probability × Impact</x:v>
+      </x:c>
+      <x:c r="B14" s="316"/>
+      <x:c r="C14" s="316"/>
+      <x:c r="D14" s="316"/>
+      <x:c r="E14" s="316"/>
+      <x:c r="F14" s="316"/>
+      <x:c r="G14" s="316"/>
+      <x:c r="H14" s="316"/>
+    </x:row>
+    <x:row r="15" ht="28" customHeight="1">
+      <x:c r="A15" s="317" t="str">
+        <x:v>Probability and Impact must each be entered as a whole number from 1 to 5. The resulting score ranges from 1 to 25.</x:v>
+      </x:c>
+      <x:c r="B15" s="317"/>
+      <x:c r="C15" s="317"/>
+      <x:c r="D15" s="317"/>
+      <x:c r="E15" s="317"/>
+      <x:c r="F15" s="317"/>
+      <x:c r="G15" s="317"/>
+      <x:c r="H15" s="317"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="315"/>
+      <x:c r="B16" s="315"/>
+      <x:c r="C16" s="315"/>
+      <x:c r="D16" s="315"/>
+      <x:c r="E16" s="315"/>
+      <x:c r="F16" s="315"/>
+      <x:c r="G16" s="315"/>
+      <x:c r="H16" s="315"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="294" t="str">
+        <x:v>RISK SCORE LEVELS</x:v>
+      </x:c>
+      <x:c r="B17" s="294"/>
+      <x:c r="C17" s="294"/>
+      <x:c r="D17" s="294"/>
+      <x:c r="E17" s="294" t="str">
+        <x:v>WORKED EXAMPLE — R1</x:v>
+      </x:c>
+      <x:c r="F17" s="294"/>
+      <x:c r="G17" s="294"/>
+      <x:c r="H17" s="294"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="318" t="str">
+        <x:v>Score</x:v>
+      </x:c>
+      <x:c r="B18" s="318" t="str">
+        <x:v>Level</x:v>
+      </x:c>
+      <x:c r="C18" s="318" t="str">
+        <x:v>Response</x:v>
+      </x:c>
+      <x:c r="D18" s="318" t="str">
+        <x:v>Suggested timing</x:v>
+      </x:c>
+      <x:c r="E18" s="319" t="str">
+        <x:v>Item</x:v>
+      </x:c>
+      <x:c r="F18" s="319" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="G18" s="319" t="str">
+        <x:v>Explanation</x:v>
+      </x:c>
+      <x:c r="H18" s="319"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="320" t="str">
+        <x:v>1–4</x:v>
+      </x:c>
+      <x:c r="B19" s="320" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="C19" s="321" t="str">
+        <x:v>Monitor and record</x:v>
+      </x:c>
+      <x:c r="D19" s="321" t="str">
+        <x:v>Routine review</x:v>
+      </x:c>
+      <x:c r="E19" s="322" t="str">
+        <x:v>Probability</x:v>
+      </x:c>
+      <x:c r="F19" s="323" t="n">
+        <x:f>'Risks'!C5</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G19" s="324" t="str">
+        <x:v>Possible</x:v>
+      </x:c>
+      <x:c r="H19" s="324"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="325" t="str">
+        <x:v>5–9</x:v>
+      </x:c>
+      <x:c r="B20" s="325" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="C20" s="326" t="str">
+        <x:v>Plan mitigation</x:v>
+      </x:c>
+      <x:c r="D20" s="326" t="str">
+        <x:v>Review regularly</x:v>
+      </x:c>
+      <x:c r="E20" s="322" t="str">
+        <x:v>Impact</x:v>
+      </x:c>
+      <x:c r="F20" s="323" t="n">
+        <x:f>'Risks'!D5</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G20" s="324" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="H20" s="324"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="327" t="str">
+        <x:v>10–14</x:v>
+      </x:c>
+      <x:c r="B21" s="327" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="C21" s="328" t="str">
+        <x:v>Mitigate and monitor closely</x:v>
+      </x:c>
+      <x:c r="D21" s="328" t="str">
+        <x:v>Prompt action</x:v>
+      </x:c>
+      <x:c r="E21" s="322" t="str">
+        <x:v>Risk Score</x:v>
+      </x:c>
+      <x:c r="F21" s="323" t="n">
+        <x:f>F19*F20</x:f>
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G21" s="324" t="str">
+        <x:v>Probability × Impact</x:v>
+      </x:c>
+      <x:c r="H21" s="324"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="329" t="str">
+        <x:v>15–25</x:v>
+      </x:c>
+      <x:c r="B22" s="329" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="C22" s="330" t="str">
+        <x:v>Escalate and act immediately</x:v>
+      </x:c>
+      <x:c r="D22" s="330" t="str">
+        <x:v>Immediate action</x:v>
+      </x:c>
+      <x:c r="E22" s="322" t="str">
+        <x:v>Risk Level</x:v>
+      </x:c>
+      <x:c r="F22" s="323" t="str">
+        <x:f>IF(F21&gt;=15,"Critical",IF(F21&gt;=10,"High",IF(F21&gt;=5,"Medium","Low")))</x:f>
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G22" s="324" t="str">
+        <x:v>Action priority</x:v>
+      </x:c>
+      <x:c r="H22" s="324"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="315"/>
+      <x:c r="B23" s="315"/>
+      <x:c r="C23" s="315"/>
+      <x:c r="D23" s="315"/>
+      <x:c r="E23" s="315"/>
+      <x:c r="F23" s="315"/>
+      <x:c r="G23" s="315"/>
+      <x:c r="H23" s="315"/>
+    </x:row>
+    <x:row r="24" ht="32" customHeight="1">
+      <x:c r="A24" s="331" t="str">
+        <x:v>Mitigation should reduce the probability, the impact, or both. Reassess the risk after controls are implemented and record the remaining (residual) risk.</x:v>
+      </x:c>
+      <x:c r="B24" s="331"/>
+      <x:c r="C24" s="331"/>
+      <x:c r="D24" s="331"/>
+      <x:c r="E24" s="331"/>
+      <x:c r="F24" s="331"/>
+      <x:c r="G24" s="331"/>
+      <x:c r="H24" s="331"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H2"/>
+    <x:mergeCell ref="A3:H3"/>
+    <x:mergeCell ref="A5:C5"/>
+    <x:mergeCell ref="D5:F5"/>
+    <x:mergeCell ref="A13:H13"/>
+    <x:mergeCell ref="A14:H14"/>
+    <x:mergeCell ref="A15:H15"/>
+    <x:mergeCell ref="A17:D17"/>
+    <x:mergeCell ref="E17:H17"/>
+    <x:mergeCell ref="A24:H24"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>